<commit_message>
add player to rr
</commit_message>
<xml_diff>
--- a/dwl-fantasy-platform/backend/WWC_Config.xlsx
+++ b/dwl-fantasy-platform/backend/WWC_Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kishan/Downloads/Delulu Leagues/DWL Delulu Women's League/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{86805392-6D4E-49F3-9229-5EF7F3965973}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2ADAD03D-6589-40CA-BDAB-6A7C1E0434ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" xr2:uid="{6957E4A2-D1A9-E849-B61B-E8AC1B9AF357}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" activeTab="5" xr2:uid="{6957E4A2-D1A9-E849-B61B-E8AC1B9AF357}"/>
   </bookViews>
   <sheets>
     <sheet name="Players" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="792" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="794" uniqueCount="226">
   <si>
     <t>Player Name</t>
   </si>
@@ -1425,7 +1425,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D6C0CFBB-B781-B648-9D72-EBCEFAF7AED5}" name="WWC_Players_All" displayName="WWC_Players_All" ref="A1:E181" totalsRowShown="0">
-  <autoFilter ref="A1:E181" xr:uid="{D6C0CFBB-B781-B648-9D72-EBCEFAF7AED5}"/>
+  <autoFilter ref="A1:E181" xr:uid="{D6C0CFBB-B781-B648-9D72-EBCEFAF7AED5}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="Rajputana Ranis"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E181">
     <sortCondition ref="A1:A181"/>
   </sortState>
@@ -1925,7 +1931,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" hidden="1">
       <c r="A2" s="14" t="s">
         <v>5</v>
       </c>
@@ -1943,7 +1949,7 @@
       </c>
       <c r="F2" s="27"/>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" hidden="1">
       <c r="A3" s="12" t="s">
         <v>9</v>
       </c>
@@ -1961,7 +1967,7 @@
       </c>
       <c r="F3" s="27"/>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" hidden="1">
       <c r="A4" s="14" t="s">
         <v>12</v>
       </c>
@@ -1979,7 +1985,7 @@
       </c>
       <c r="F4" s="27"/>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" hidden="1">
       <c r="A5" s="12" t="s">
         <v>14</v>
       </c>
@@ -1993,7 +1999,7 @@
       <c r="E5" s="26"/>
       <c r="F5" s="27"/>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" hidden="1">
       <c r="A6" s="8" t="s">
         <v>16</v>
       </c>
@@ -2007,7 +2013,7 @@
       <c r="E6" s="26"/>
       <c r="F6" s="27"/>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" hidden="1">
       <c r="A7" s="8" t="s">
         <v>18</v>
       </c>
@@ -2021,7 +2027,7 @@
       <c r="E7" s="26"/>
       <c r="F7" s="27"/>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" hidden="1">
       <c r="A8" s="4" t="s">
         <v>19</v>
       </c>
@@ -2057,7 +2063,7 @@
       </c>
       <c r="F9" s="27"/>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" hidden="1">
       <c r="A10" s="11" t="s">
         <v>25</v>
       </c>
@@ -2071,7 +2077,7 @@
       <c r="E10" s="26"/>
       <c r="F10" s="27"/>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" hidden="1">
       <c r="A11" s="8" t="s">
         <v>27</v>
       </c>
@@ -2089,7 +2095,7 @@
       </c>
       <c r="F11" s="27"/>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" hidden="1">
       <c r="A12" s="6" t="s">
         <v>28</v>
       </c>
@@ -2107,7 +2113,7 @@
       </c>
       <c r="F12" s="27"/>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" hidden="1">
       <c r="A13" s="4" t="s">
         <v>30</v>
       </c>
@@ -2125,7 +2131,7 @@
       </c>
       <c r="F13" s="27"/>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" hidden="1">
       <c r="A14" s="13" t="s">
         <v>31</v>
       </c>
@@ -2143,7 +2149,7 @@
       </c>
       <c r="F14" s="27"/>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" hidden="1">
       <c r="A15" s="8" t="s">
         <v>33</v>
       </c>
@@ -2175,7 +2181,7 @@
       </c>
       <c r="F16" s="27"/>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" hidden="1">
       <c r="A17" s="4" t="s">
         <v>36</v>
       </c>
@@ -2193,7 +2199,7 @@
       </c>
       <c r="F17" s="27"/>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" hidden="1">
       <c r="A18" s="14" t="s">
         <v>38</v>
       </c>
@@ -2207,7 +2213,7 @@
       <c r="E18" s="26"/>
       <c r="F18" s="27"/>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" hidden="1">
       <c r="A19" s="8" t="s">
         <v>39</v>
       </c>
@@ -2239,7 +2245,7 @@
       </c>
       <c r="F20" s="27"/>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" hidden="1">
       <c r="A21" s="11" t="s">
         <v>41</v>
       </c>
@@ -2257,7 +2263,7 @@
       </c>
       <c r="F21" s="27"/>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" hidden="1">
       <c r="A22" s="9" t="s">
         <v>43</v>
       </c>
@@ -2271,7 +2277,7 @@
       <c r="E22" s="26"/>
       <c r="F22" s="27"/>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" hidden="1">
       <c r="A23" s="4" t="s">
         <v>45</v>
       </c>
@@ -2289,7 +2295,7 @@
       </c>
       <c r="F23" s="27"/>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" hidden="1">
       <c r="A24" s="7" t="s">
         <v>46</v>
       </c>
@@ -2307,7 +2313,7 @@
       </c>
       <c r="F24" s="27"/>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" hidden="1">
       <c r="A25" s="10" t="s">
         <v>47</v>
       </c>
@@ -2325,7 +2331,7 @@
       </c>
       <c r="F25" s="27"/>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" hidden="1">
       <c r="A26" s="10" t="s">
         <v>49</v>
       </c>
@@ -2343,7 +2349,7 @@
       </c>
       <c r="F26" s="27"/>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" hidden="1">
       <c r="A27" s="8" t="s">
         <v>50</v>
       </c>
@@ -2361,7 +2367,7 @@
       </c>
       <c r="F27" s="27"/>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:6" hidden="1">
       <c r="A28" s="9" t="s">
         <v>51</v>
       </c>
@@ -2393,7 +2399,7 @@
       </c>
       <c r="F29" s="27"/>
     </row>
-    <row r="30" spans="1:6">
+    <row r="30" spans="1:6" hidden="1">
       <c r="A30" s="6" t="s">
         <v>54</v>
       </c>
@@ -2411,7 +2417,7 @@
       </c>
       <c r="F30" s="27"/>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" hidden="1">
       <c r="A31" s="14" t="s">
         <v>55</v>
       </c>
@@ -2429,7 +2435,7 @@
       </c>
       <c r="F31" s="27"/>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:6" hidden="1">
       <c r="A32" s="12" t="s">
         <v>57</v>
       </c>
@@ -2443,7 +2449,7 @@
       <c r="E32" s="26"/>
       <c r="F32" s="27"/>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:6" hidden="1">
       <c r="A33" s="13" t="s">
         <v>58</v>
       </c>
@@ -2461,7 +2467,7 @@
       </c>
       <c r="F33" s="27"/>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:6" hidden="1">
       <c r="A34" s="8" t="s">
         <v>59</v>
       </c>
@@ -2475,7 +2481,7 @@
       <c r="E34" s="26"/>
       <c r="F34" s="27"/>
     </row>
-    <row r="35" spans="1:6">
+    <row r="35" spans="1:6" hidden="1">
       <c r="A35" s="13" t="s">
         <v>60</v>
       </c>
@@ -2493,7 +2499,7 @@
       </c>
       <c r="F35" s="27"/>
     </row>
-    <row r="36" spans="1:6">
+    <row r="36" spans="1:6" hidden="1">
       <c r="A36" s="6" t="s">
         <v>61</v>
       </c>
@@ -2507,7 +2513,7 @@
       <c r="E36" s="26"/>
       <c r="F36" s="27"/>
     </row>
-    <row r="37" spans="1:6">
+    <row r="37" spans="1:6" hidden="1">
       <c r="A37" s="6" t="s">
         <v>62</v>
       </c>
@@ -2525,7 +2531,7 @@
       </c>
       <c r="F37" s="27"/>
     </row>
-    <row r="38" spans="1:6">
+    <row r="38" spans="1:6" hidden="1">
       <c r="A38" s="12" t="s">
         <v>63</v>
       </c>
@@ -2539,7 +2545,7 @@
       <c r="E38" s="26"/>
       <c r="F38" s="27"/>
     </row>
-    <row r="39" spans="1:6">
+    <row r="39" spans="1:6" hidden="1">
       <c r="A39" s="14" t="s">
         <v>64</v>
       </c>
@@ -2557,7 +2563,7 @@
       </c>
       <c r="F39" s="27"/>
     </row>
-    <row r="40" spans="1:6">
+    <row r="40" spans="1:6" hidden="1">
       <c r="A40" s="7" t="s">
         <v>65</v>
       </c>
@@ -2575,7 +2581,7 @@
       </c>
       <c r="F40" s="27"/>
     </row>
-    <row r="41" spans="1:6">
+    <row r="41" spans="1:6" hidden="1">
       <c r="A41" s="11" t="s">
         <v>66</v>
       </c>
@@ -2589,7 +2595,7 @@
       <c r="E41" s="26"/>
       <c r="F41" s="27"/>
     </row>
-    <row r="42" spans="1:6">
+    <row r="42" spans="1:6" hidden="1">
       <c r="A42" s="5" t="s">
         <v>67</v>
       </c>
@@ -2603,7 +2609,7 @@
       <c r="E42" s="26"/>
       <c r="F42" s="27"/>
     </row>
-    <row r="43" spans="1:6">
+    <row r="43" spans="1:6" hidden="1">
       <c r="A43" s="4" t="s">
         <v>69</v>
       </c>
@@ -2621,7 +2627,7 @@
       </c>
       <c r="F43" s="27"/>
     </row>
-    <row r="44" spans="1:6">
+    <row r="44" spans="1:6" hidden="1">
       <c r="A44" s="11" t="s">
         <v>70</v>
       </c>
@@ -2635,7 +2641,7 @@
       <c r="E44" s="26"/>
       <c r="F44" s="27"/>
     </row>
-    <row r="45" spans="1:6">
+    <row r="45" spans="1:6" hidden="1">
       <c r="A45" s="5" t="s">
         <v>71</v>
       </c>
@@ -2649,7 +2655,7 @@
       <c r="E45" s="26"/>
       <c r="F45" s="27"/>
     </row>
-    <row r="46" spans="1:6">
+    <row r="46" spans="1:6" hidden="1">
       <c r="A46" s="5" t="s">
         <v>72</v>
       </c>
@@ -2663,7 +2669,7 @@
       <c r="E46" s="26"/>
       <c r="F46" s="27"/>
     </row>
-    <row r="47" spans="1:6">
+    <row r="47" spans="1:6" hidden="1">
       <c r="A47" s="11" t="s">
         <v>73</v>
       </c>
@@ -2681,7 +2687,7 @@
       </c>
       <c r="F47" s="27"/>
     </row>
-    <row r="48" spans="1:6">
+    <row r="48" spans="1:6" hidden="1">
       <c r="A48" s="10" t="s">
         <v>74</v>
       </c>
@@ -2695,7 +2701,7 @@
       <c r="E48" s="26"/>
       <c r="F48" s="27"/>
     </row>
-    <row r="49" spans="1:6">
+    <row r="49" spans="1:6" hidden="1">
       <c r="A49" s="9" t="s">
         <v>75</v>
       </c>
@@ -2709,7 +2715,7 @@
       <c r="E49" s="26"/>
       <c r="F49" s="27"/>
     </row>
-    <row r="50" spans="1:6">
+    <row r="50" spans="1:6" hidden="1">
       <c r="A50" s="6" t="s">
         <v>76</v>
       </c>
@@ -2727,7 +2733,7 @@
       </c>
       <c r="F50" s="27"/>
     </row>
-    <row r="51" spans="1:6">
+    <row r="51" spans="1:6" hidden="1">
       <c r="A51" s="12" t="s">
         <v>77</v>
       </c>
@@ -2739,7 +2745,7 @@
       <c r="E51" s="26"/>
       <c r="F51" s="27"/>
     </row>
-    <row r="52" spans="1:6">
+    <row r="52" spans="1:6" hidden="1">
       <c r="A52" s="8" t="s">
         <v>78</v>
       </c>
@@ -2757,7 +2763,7 @@
       </c>
       <c r="F52" s="27"/>
     </row>
-    <row r="53" spans="1:6">
+    <row r="53" spans="1:6" hidden="1">
       <c r="A53" s="10" t="s">
         <v>79</v>
       </c>
@@ -2811,7 +2817,7 @@
       </c>
       <c r="F55" s="27"/>
     </row>
-    <row r="56" spans="1:6">
+    <row r="56" spans="1:6" hidden="1">
       <c r="A56" s="8" t="s">
         <v>82</v>
       </c>
@@ -2825,7 +2831,7 @@
       <c r="E56" s="26"/>
       <c r="F56" s="27"/>
     </row>
-    <row r="57" spans="1:6">
+    <row r="57" spans="1:6" hidden="1">
       <c r="A57" s="4" t="s">
         <v>83</v>
       </c>
@@ -2843,7 +2849,7 @@
       </c>
       <c r="F57" s="27"/>
     </row>
-    <row r="58" spans="1:6">
+    <row r="58" spans="1:6" hidden="1">
       <c r="A58" s="11" t="s">
         <v>84</v>
       </c>
@@ -2857,7 +2863,7 @@
       <c r="E58" s="26"/>
       <c r="F58" s="27"/>
     </row>
-    <row r="59" spans="1:6">
+    <row r="59" spans="1:6" hidden="1">
       <c r="A59" s="9" t="s">
         <v>85</v>
       </c>
@@ -2871,7 +2877,7 @@
       <c r="E59" s="26"/>
       <c r="F59" s="27"/>
     </row>
-    <row r="60" spans="1:6">
+    <row r="60" spans="1:6" hidden="1">
       <c r="A60" s="15" t="s">
         <v>86</v>
       </c>
@@ -2885,7 +2891,7 @@
       <c r="E60" s="26"/>
       <c r="F60" s="27"/>
     </row>
-    <row r="61" spans="1:6">
+    <row r="61" spans="1:6" hidden="1">
       <c r="A61" s="7" t="s">
         <v>87</v>
       </c>
@@ -2903,7 +2909,7 @@
       </c>
       <c r="F61" s="27"/>
     </row>
-    <row r="62" spans="1:6">
+    <row r="62" spans="1:6" hidden="1">
       <c r="A62" s="15" t="s">
         <v>88</v>
       </c>
@@ -2921,7 +2927,7 @@
       </c>
       <c r="F62" s="27"/>
     </row>
-    <row r="63" spans="1:6">
+    <row r="63" spans="1:6" hidden="1">
       <c r="A63" s="15" t="s">
         <v>89</v>
       </c>
@@ -2935,7 +2941,7 @@
       <c r="E63" s="26"/>
       <c r="F63" s="27"/>
     </row>
-    <row r="64" spans="1:6">
+    <row r="64" spans="1:6" hidden="1">
       <c r="A64" s="14" t="s">
         <v>90</v>
       </c>
@@ -2953,7 +2959,7 @@
       </c>
       <c r="F64" s="27"/>
     </row>
-    <row r="65" spans="1:6">
+    <row r="65" spans="1:6" hidden="1">
       <c r="A65" s="6" t="s">
         <v>91</v>
       </c>
@@ -2971,7 +2977,7 @@
       </c>
       <c r="F65" s="27"/>
     </row>
-    <row r="66" spans="1:6">
+    <row r="66" spans="1:6" hidden="1">
       <c r="A66" s="9" t="s">
         <v>92</v>
       </c>
@@ -2985,7 +2991,7 @@
       <c r="E66" s="26"/>
       <c r="F66" s="27"/>
     </row>
-    <row r="67" spans="1:6">
+    <row r="67" spans="1:6" hidden="1">
       <c r="A67" s="15" t="s">
         <v>93</v>
       </c>
@@ -2999,7 +3005,7 @@
       <c r="E67" s="26"/>
       <c r="F67" s="27"/>
     </row>
-    <row r="68" spans="1:6">
+    <row r="68" spans="1:6" hidden="1">
       <c r="A68" s="11" t="s">
         <v>94</v>
       </c>
@@ -3013,7 +3019,7 @@
       <c r="E68" s="26"/>
       <c r="F68" s="27"/>
     </row>
-    <row r="69" spans="1:6">
+    <row r="69" spans="1:6" hidden="1">
       <c r="A69" s="9" t="s">
         <v>95</v>
       </c>
@@ -3027,7 +3033,7 @@
       <c r="E69" s="26"/>
       <c r="F69" s="27"/>
     </row>
-    <row r="70" spans="1:6">
+    <row r="70" spans="1:6" hidden="1">
       <c r="A70" s="9" t="s">
         <v>96</v>
       </c>
@@ -3041,7 +3047,7 @@
       <c r="E70" s="26"/>
       <c r="F70" s="27"/>
     </row>
-    <row r="71" spans="1:6">
+    <row r="71" spans="1:6" hidden="1">
       <c r="A71" s="10" t="s">
         <v>97</v>
       </c>
@@ -3055,7 +3061,7 @@
       <c r="E71" s="26"/>
       <c r="F71" s="27"/>
     </row>
-    <row r="72" spans="1:6">
+    <row r="72" spans="1:6" hidden="1">
       <c r="A72" s="6" t="s">
         <v>98</v>
       </c>
@@ -3073,7 +3079,7 @@
       </c>
       <c r="F72" s="27"/>
     </row>
-    <row r="73" spans="1:6">
+    <row r="73" spans="1:6" hidden="1">
       <c r="A73" s="10" t="s">
         <v>99</v>
       </c>
@@ -3091,7 +3097,7 @@
       </c>
       <c r="F73" s="27"/>
     </row>
-    <row r="74" spans="1:6">
+    <row r="74" spans="1:6" hidden="1">
       <c r="A74" s="14" t="s">
         <v>100</v>
       </c>
@@ -3105,7 +3111,7 @@
       <c r="E74" s="26"/>
       <c r="F74" s="27"/>
     </row>
-    <row r="75" spans="1:6">
+    <row r="75" spans="1:6" hidden="1">
       <c r="A75" s="14" t="s">
         <v>101</v>
       </c>
@@ -3155,7 +3161,7 @@
       </c>
       <c r="F77" s="27"/>
     </row>
-    <row r="78" spans="1:6">
+    <row r="78" spans="1:6" hidden="1">
       <c r="A78" s="5" t="s">
         <v>104</v>
       </c>
@@ -3169,7 +3175,7 @@
       <c r="E78" s="26"/>
       <c r="F78" s="27"/>
     </row>
-    <row r="79" spans="1:6">
+    <row r="79" spans="1:6" hidden="1">
       <c r="A79" s="13" t="s">
         <v>105</v>
       </c>
@@ -3187,7 +3193,7 @@
       </c>
       <c r="F79" s="27"/>
     </row>
-    <row r="80" spans="1:6">
+    <row r="80" spans="1:6" hidden="1">
       <c r="A80" s="14" t="s">
         <v>106</v>
       </c>
@@ -3205,7 +3211,7 @@
       </c>
       <c r="F80" s="27"/>
     </row>
-    <row r="81" spans="1:6">
+    <row r="81" spans="1:6" hidden="1">
       <c r="A81" s="12" t="s">
         <v>107</v>
       </c>
@@ -3219,7 +3225,7 @@
       <c r="E81" s="26"/>
       <c r="F81" s="27"/>
     </row>
-    <row r="82" spans="1:6">
+    <row r="82" spans="1:6" hidden="1">
       <c r="A82" s="12" t="s">
         <v>108</v>
       </c>
@@ -3237,7 +3243,7 @@
       </c>
       <c r="F82" s="27"/>
     </row>
-    <row r="83" spans="1:6">
+    <row r="83" spans="1:6" hidden="1">
       <c r="A83" s="15" t="s">
         <v>109</v>
       </c>
@@ -3251,7 +3257,7 @@
       <c r="E83" s="26"/>
       <c r="F83" s="27"/>
     </row>
-    <row r="84" spans="1:6">
+    <row r="84" spans="1:6" hidden="1">
       <c r="A84" s="15" t="s">
         <v>110</v>
       </c>
@@ -3265,7 +3271,7 @@
       <c r="E84" s="26"/>
       <c r="F84" s="27"/>
     </row>
-    <row r="85" spans="1:6">
+    <row r="85" spans="1:6" hidden="1">
       <c r="A85" s="15" t="s">
         <v>111</v>
       </c>
@@ -3279,7 +3285,7 @@
       <c r="E85" s="26"/>
       <c r="F85" s="27"/>
     </row>
-    <row r="86" spans="1:6">
+    <row r="86" spans="1:6" hidden="1">
       <c r="A86" s="13" t="s">
         <v>112</v>
       </c>
@@ -3297,7 +3303,7 @@
       </c>
       <c r="F86" s="27"/>
     </row>
-    <row r="87" spans="1:6">
+    <row r="87" spans="1:6" hidden="1">
       <c r="A87" s="4" t="s">
         <v>113</v>
       </c>
@@ -3315,7 +3321,7 @@
       </c>
       <c r="F87" s="27"/>
     </row>
-    <row r="88" spans="1:6">
+    <row r="88" spans="1:6" hidden="1">
       <c r="A88" s="12" t="s">
         <v>114</v>
       </c>
@@ -3347,7 +3353,7 @@
       </c>
       <c r="F89" s="27"/>
     </row>
-    <row r="90" spans="1:6">
+    <row r="90" spans="1:6" hidden="1">
       <c r="A90" s="9" t="s">
         <v>116</v>
       </c>
@@ -3361,7 +3367,7 @@
       <c r="E90" s="26"/>
       <c r="F90" s="27"/>
     </row>
-    <row r="91" spans="1:6">
+    <row r="91" spans="1:6" hidden="1">
       <c r="A91" s="8" t="s">
         <v>117</v>
       </c>
@@ -3373,7 +3379,7 @@
       <c r="E91" s="26"/>
       <c r="F91" s="27"/>
     </row>
-    <row r="92" spans="1:6">
+    <row r="92" spans="1:6" hidden="1">
       <c r="A92" s="8" t="s">
         <v>118</v>
       </c>
@@ -3387,7 +3393,7 @@
       <c r="E92" s="26"/>
       <c r="F92" s="27"/>
     </row>
-    <row r="93" spans="1:6">
+    <row r="93" spans="1:6" hidden="1">
       <c r="A93" s="13" t="s">
         <v>119</v>
       </c>
@@ -3405,7 +3411,7 @@
       </c>
       <c r="F93" s="27"/>
     </row>
-    <row r="94" spans="1:6">
+    <row r="94" spans="1:6" hidden="1">
       <c r="A94" s="6" t="s">
         <v>120</v>
       </c>
@@ -3423,7 +3429,7 @@
       </c>
       <c r="F94" s="27"/>
     </row>
-    <row r="95" spans="1:6">
+    <row r="95" spans="1:6" hidden="1">
       <c r="A95" s="6" t="s">
         <v>121</v>
       </c>
@@ -3441,7 +3447,7 @@
       </c>
       <c r="F95" s="27"/>
     </row>
-    <row r="96" spans="1:6">
+    <row r="96" spans="1:6" hidden="1">
       <c r="A96" s="10" t="s">
         <v>122</v>
       </c>
@@ -3459,7 +3465,7 @@
       </c>
       <c r="F96" s="27"/>
     </row>
-    <row r="97" spans="1:6">
+    <row r="97" spans="1:6" hidden="1">
       <c r="A97" s="8" t="s">
         <v>123</v>
       </c>
@@ -3477,7 +3483,7 @@
       </c>
       <c r="F97" s="27"/>
     </row>
-    <row r="98" spans="1:6">
+    <row r="98" spans="1:6" hidden="1">
       <c r="A98" s="6" t="s">
         <v>124</v>
       </c>
@@ -3495,7 +3501,7 @@
       </c>
       <c r="F98" s="27"/>
     </row>
-    <row r="99" spans="1:6">
+    <row r="99" spans="1:6" hidden="1">
       <c r="A99" s="8" t="s">
         <v>125</v>
       </c>
@@ -3509,7 +3515,7 @@
       <c r="E99" s="26"/>
       <c r="F99" s="27"/>
     </row>
-    <row r="100" spans="1:6">
+    <row r="100" spans="1:6" hidden="1">
       <c r="A100" s="4" t="s">
         <v>126</v>
       </c>
@@ -3527,7 +3533,7 @@
       </c>
       <c r="F100" s="27"/>
     </row>
-    <row r="101" spans="1:6">
+    <row r="101" spans="1:6" hidden="1">
       <c r="A101" s="10" t="s">
         <v>127</v>
       </c>
@@ -3541,7 +3547,7 @@
       <c r="E101" s="26"/>
       <c r="F101" s="27"/>
     </row>
-    <row r="102" spans="1:6">
+    <row r="102" spans="1:6" hidden="1">
       <c r="A102" s="12" t="s">
         <v>128</v>
       </c>
@@ -3555,7 +3561,7 @@
       <c r="E102" s="26"/>
       <c r="F102" s="27"/>
     </row>
-    <row r="103" spans="1:6">
+    <row r="103" spans="1:6" hidden="1">
       <c r="A103" s="15" t="s">
         <v>129</v>
       </c>
@@ -3569,7 +3575,7 @@
       <c r="E103" s="26"/>
       <c r="F103" s="27"/>
     </row>
-    <row r="104" spans="1:6">
+    <row r="104" spans="1:6" hidden="1">
       <c r="A104" s="14" t="s">
         <v>130</v>
       </c>
@@ -3583,7 +3589,7 @@
       <c r="E104" s="26"/>
       <c r="F104" s="27"/>
     </row>
-    <row r="105" spans="1:6">
+    <row r="105" spans="1:6" hidden="1">
       <c r="A105" s="13" t="s">
         <v>131</v>
       </c>
@@ -3601,7 +3607,7 @@
       </c>
       <c r="F105" s="27"/>
     </row>
-    <row r="106" spans="1:6">
+    <row r="106" spans="1:6" hidden="1">
       <c r="A106" s="5" t="s">
         <v>132</v>
       </c>
@@ -3615,7 +3621,7 @@
       <c r="E106" s="26"/>
       <c r="F106" s="27"/>
     </row>
-    <row r="107" spans="1:6">
+    <row r="107" spans="1:6" hidden="1">
       <c r="A107" s="12" t="s">
         <v>133</v>
       </c>
@@ -3629,7 +3635,7 @@
       <c r="E107" s="26"/>
       <c r="F107" s="27"/>
     </row>
-    <row r="108" spans="1:6">
+    <row r="108" spans="1:6" hidden="1">
       <c r="A108" s="4" t="s">
         <v>134</v>
       </c>
@@ -3647,7 +3653,7 @@
       </c>
       <c r="F108" s="27"/>
     </row>
-    <row r="109" spans="1:6">
+    <row r="109" spans="1:6" hidden="1">
       <c r="A109" s="10" t="s">
         <v>135</v>
       </c>
@@ -3665,7 +3671,7 @@
       </c>
       <c r="F109" s="27"/>
     </row>
-    <row r="110" spans="1:6">
+    <row r="110" spans="1:6" hidden="1">
       <c r="A110" s="15" t="s">
         <v>136</v>
       </c>
@@ -3679,7 +3685,7 @@
       <c r="E110" s="26"/>
       <c r="F110" s="27"/>
     </row>
-    <row r="111" spans="1:6">
+    <row r="111" spans="1:6" hidden="1">
       <c r="A111" s="11" t="s">
         <v>137</v>
       </c>
@@ -3697,7 +3703,7 @@
       </c>
       <c r="F111" s="27"/>
     </row>
-    <row r="112" spans="1:6">
+    <row r="112" spans="1:6" hidden="1">
       <c r="A112" s="9" t="s">
         <v>138</v>
       </c>
@@ -3711,7 +3717,7 @@
       <c r="E112" s="26"/>
       <c r="F112" s="27"/>
     </row>
-    <row r="113" spans="1:6">
+    <row r="113" spans="1:6" hidden="1">
       <c r="A113" s="13" t="s">
         <v>139</v>
       </c>
@@ -3729,7 +3735,7 @@
       </c>
       <c r="F113" s="27"/>
     </row>
-    <row r="114" spans="1:6">
+    <row r="114" spans="1:6" hidden="1">
       <c r="A114" s="5" t="s">
         <v>140</v>
       </c>
@@ -3747,7 +3753,7 @@
       </c>
       <c r="F114" s="27"/>
     </row>
-    <row r="115" spans="1:6">
+    <row r="115" spans="1:6" hidden="1">
       <c r="A115" s="7" t="s">
         <v>141</v>
       </c>
@@ -3775,11 +3781,15 @@
       <c r="C116" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="D116" s="11"/>
-      <c r="E116" s="26"/>
+      <c r="D116" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="E116" s="26">
+        <v>7</v>
+      </c>
       <c r="F116" s="27"/>
     </row>
-    <row r="117" spans="1:6">
+    <row r="117" spans="1:6" hidden="1">
       <c r="A117" s="6" t="s">
         <v>143</v>
       </c>
@@ -3797,7 +3807,7 @@
       </c>
       <c r="F117" s="27"/>
     </row>
-    <row r="118" spans="1:6">
+    <row r="118" spans="1:6" hidden="1">
       <c r="A118" s="11" t="s">
         <v>144</v>
       </c>
@@ -3811,7 +3821,7 @@
       <c r="E118" s="26"/>
       <c r="F118" s="27"/>
     </row>
-    <row r="119" spans="1:6">
+    <row r="119" spans="1:6" hidden="1">
       <c r="A119" s="10" t="s">
         <v>145</v>
       </c>
@@ -3825,7 +3835,7 @@
       <c r="E119" s="26"/>
       <c r="F119" s="27"/>
     </row>
-    <row r="120" spans="1:6">
+    <row r="120" spans="1:6" hidden="1">
       <c r="A120" s="4" t="s">
         <v>146</v>
       </c>
@@ -3843,7 +3853,7 @@
       </c>
       <c r="F120" s="27"/>
     </row>
-    <row r="121" spans="1:6">
+    <row r="121" spans="1:6" hidden="1">
       <c r="A121" s="5" t="s">
         <v>147</v>
       </c>
@@ -3861,7 +3871,7 @@
       </c>
       <c r="F121" s="27"/>
     </row>
-    <row r="122" spans="1:6">
+    <row r="122" spans="1:6" hidden="1">
       <c r="A122" s="15" t="s">
         <v>148</v>
       </c>
@@ -3875,7 +3885,7 @@
       <c r="E122" s="26"/>
       <c r="F122" s="27"/>
     </row>
-    <row r="123" spans="1:6">
+    <row r="123" spans="1:6" hidden="1">
       <c r="A123" s="15" t="s">
         <v>149</v>
       </c>
@@ -3889,7 +3899,7 @@
       <c r="E123" s="26"/>
       <c r="F123" s="27"/>
     </row>
-    <row r="124" spans="1:6">
+    <row r="124" spans="1:6" hidden="1">
       <c r="A124" s="13" t="s">
         <v>150</v>
       </c>
@@ -3907,7 +3917,7 @@
       </c>
       <c r="F124" s="27"/>
     </row>
-    <row r="125" spans="1:6">
+    <row r="125" spans="1:6" hidden="1">
       <c r="A125" s="12" t="s">
         <v>151</v>
       </c>
@@ -3921,7 +3931,7 @@
       <c r="E125" s="26"/>
       <c r="F125" s="27"/>
     </row>
-    <row r="126" spans="1:6">
+    <row r="126" spans="1:6" hidden="1">
       <c r="A126" s="8" t="s">
         <v>152</v>
       </c>
@@ -3939,7 +3949,7 @@
       </c>
       <c r="F126" s="27"/>
     </row>
-    <row r="127" spans="1:6">
+    <row r="127" spans="1:6" hidden="1">
       <c r="A127" s="9" t="s">
         <v>153</v>
       </c>
@@ -3953,7 +3963,7 @@
       <c r="E127" s="26"/>
       <c r="F127" s="27"/>
     </row>
-    <row r="128" spans="1:6">
+    <row r="128" spans="1:6" hidden="1">
       <c r="A128" s="4" t="s">
         <v>154</v>
       </c>
@@ -3971,7 +3981,7 @@
       </c>
       <c r="F128" s="27"/>
     </row>
-    <row r="129" spans="1:6">
+    <row r="129" spans="1:6" hidden="1">
       <c r="A129" s="12" t="s">
         <v>155</v>
       </c>
@@ -3989,7 +3999,7 @@
       </c>
       <c r="F129" s="27"/>
     </row>
-    <row r="130" spans="1:6">
+    <row r="130" spans="1:6" hidden="1">
       <c r="A130" s="10" t="s">
         <v>156</v>
       </c>
@@ -4007,7 +4017,7 @@
       </c>
       <c r="F130" s="27"/>
     </row>
-    <row r="131" spans="1:6">
+    <row r="131" spans="1:6" hidden="1">
       <c r="A131" s="12" t="s">
         <v>157</v>
       </c>
@@ -4021,7 +4031,7 @@
       <c r="E131" s="26"/>
       <c r="F131" s="27"/>
     </row>
-    <row r="132" spans="1:6">
+    <row r="132" spans="1:6" hidden="1">
       <c r="A132" s="14" t="s">
         <v>158</v>
       </c>
@@ -4035,7 +4045,7 @@
       <c r="E132" s="26"/>
       <c r="F132" s="27"/>
     </row>
-    <row r="133" spans="1:6">
+    <row r="133" spans="1:6" hidden="1">
       <c r="A133" s="5" t="s">
         <v>159</v>
       </c>
@@ -4049,7 +4059,7 @@
       <c r="E133" s="26"/>
       <c r="F133" s="27"/>
     </row>
-    <row r="134" spans="1:6">
+    <row r="134" spans="1:6" hidden="1">
       <c r="A134" s="12" t="s">
         <v>160</v>
       </c>
@@ -4063,7 +4073,7 @@
       <c r="E134" s="26"/>
       <c r="F134" s="27"/>
     </row>
-    <row r="135" spans="1:6">
+    <row r="135" spans="1:6" hidden="1">
       <c r="A135" s="7" t="s">
         <v>161</v>
       </c>
@@ -4081,7 +4091,7 @@
       </c>
       <c r="F135" s="27"/>
     </row>
-    <row r="136" spans="1:6">
+    <row r="136" spans="1:6" hidden="1">
       <c r="A136" s="11" t="s">
         <v>162</v>
       </c>
@@ -4095,7 +4105,7 @@
       <c r="E136" s="26"/>
       <c r="F136" s="27"/>
     </row>
-    <row r="137" spans="1:6">
+    <row r="137" spans="1:6" hidden="1">
       <c r="A137" s="8" t="s">
         <v>163</v>
       </c>
@@ -4109,7 +4119,7 @@
       <c r="E137" s="26"/>
       <c r="F137" s="27"/>
     </row>
-    <row r="138" spans="1:6">
+    <row r="138" spans="1:6" hidden="1">
       <c r="A138" s="7" t="s">
         <v>164</v>
       </c>
@@ -4127,7 +4137,7 @@
       </c>
       <c r="F138" s="27"/>
     </row>
-    <row r="139" spans="1:6">
+    <row r="139" spans="1:6" hidden="1">
       <c r="A139" s="7" t="s">
         <v>165</v>
       </c>
@@ -4145,7 +4155,7 @@
       </c>
       <c r="F139" s="27"/>
     </row>
-    <row r="140" spans="1:6">
+    <row r="140" spans="1:6" hidden="1">
       <c r="A140" s="5" t="s">
         <v>166</v>
       </c>
@@ -4159,7 +4169,7 @@
       <c r="E140" s="26"/>
       <c r="F140" s="27"/>
     </row>
-    <row r="141" spans="1:6">
+    <row r="141" spans="1:6" hidden="1">
       <c r="A141" s="9" t="s">
         <v>167</v>
       </c>
@@ -4177,7 +4187,7 @@
       </c>
       <c r="F141" s="27"/>
     </row>
-    <row r="142" spans="1:6">
+    <row r="142" spans="1:6" hidden="1">
       <c r="A142" s="9" t="s">
         <v>168</v>
       </c>
@@ -4191,7 +4201,7 @@
       <c r="E142" s="26"/>
       <c r="F142" s="27"/>
     </row>
-    <row r="143" spans="1:6">
+    <row r="143" spans="1:6" hidden="1">
       <c r="A143" s="10" t="s">
         <v>169</v>
       </c>
@@ -4209,7 +4219,7 @@
       </c>
       <c r="F143" s="27"/>
     </row>
-    <row r="144" spans="1:6">
+    <row r="144" spans="1:6" hidden="1">
       <c r="A144" s="11" t="s">
         <v>170</v>
       </c>
@@ -4227,7 +4237,7 @@
       </c>
       <c r="F144" s="27"/>
     </row>
-    <row r="145" spans="1:6">
+    <row r="145" spans="1:6" hidden="1">
       <c r="A145" s="11" t="s">
         <v>171</v>
       </c>
@@ -4241,7 +4251,7 @@
       <c r="E145" s="26"/>
       <c r="F145" s="27"/>
     </row>
-    <row r="146" spans="1:6">
+    <row r="146" spans="1:6" hidden="1">
       <c r="A146" s="9" t="s">
         <v>172</v>
       </c>
@@ -4255,7 +4265,7 @@
       <c r="E146" s="26"/>
       <c r="F146" s="27"/>
     </row>
-    <row r="147" spans="1:6">
+    <row r="147" spans="1:6" hidden="1">
       <c r="A147" s="12" t="s">
         <v>173</v>
       </c>
@@ -4291,7 +4301,7 @@
       </c>
       <c r="F148" s="27"/>
     </row>
-    <row r="149" spans="1:6">
+    <row r="149" spans="1:6" hidden="1">
       <c r="A149" s="7" t="s">
         <v>175</v>
       </c>
@@ -4309,7 +4319,7 @@
       </c>
       <c r="F149" s="27"/>
     </row>
-    <row r="150" spans="1:6">
+    <row r="150" spans="1:6" hidden="1">
       <c r="A150" s="5" t="s">
         <v>176</v>
       </c>
@@ -4323,7 +4333,7 @@
       <c r="E150" s="26"/>
       <c r="F150" s="27"/>
     </row>
-    <row r="151" spans="1:6">
+    <row r="151" spans="1:6" hidden="1">
       <c r="A151" s="15" t="s">
         <v>177</v>
       </c>
@@ -4337,7 +4347,7 @@
       <c r="E151" s="26"/>
       <c r="F151" s="27"/>
     </row>
-    <row r="152" spans="1:6">
+    <row r="152" spans="1:6" hidden="1">
       <c r="A152" s="14" t="s">
         <v>178</v>
       </c>
@@ -4351,7 +4361,7 @@
       <c r="E152" s="26"/>
       <c r="F152" s="27"/>
     </row>
-    <row r="153" spans="1:6">
+    <row r="153" spans="1:6" hidden="1">
       <c r="A153" s="14" t="s">
         <v>179</v>
       </c>
@@ -4369,7 +4379,7 @@
       </c>
       <c r="F153" s="27"/>
     </row>
-    <row r="154" spans="1:6">
+    <row r="154" spans="1:6" hidden="1">
       <c r="A154" s="5" t="s">
         <v>180</v>
       </c>
@@ -4383,7 +4393,7 @@
       <c r="E154" s="26"/>
       <c r="F154" s="27"/>
     </row>
-    <row r="155" spans="1:6">
+    <row r="155" spans="1:6" hidden="1">
       <c r="A155" s="7" t="s">
         <v>181</v>
       </c>
@@ -4401,7 +4411,7 @@
       </c>
       <c r="F155" s="27"/>
     </row>
-    <row r="156" spans="1:6">
+    <row r="156" spans="1:6" hidden="1">
       <c r="A156" s="7" t="s">
         <v>182</v>
       </c>
@@ -4419,7 +4429,7 @@
       </c>
       <c r="F156" s="27"/>
     </row>
-    <row r="157" spans="1:6">
+    <row r="157" spans="1:6" hidden="1">
       <c r="A157" s="9" t="s">
         <v>183</v>
       </c>
@@ -4433,7 +4443,7 @@
       <c r="E157" s="26"/>
       <c r="F157" s="27"/>
     </row>
-    <row r="158" spans="1:6">
+    <row r="158" spans="1:6" hidden="1">
       <c r="A158" s="13" t="s">
         <v>184</v>
       </c>
@@ -4451,7 +4461,7 @@
       </c>
       <c r="F158" s="27"/>
     </row>
-    <row r="159" spans="1:6">
+    <row r="159" spans="1:6" hidden="1">
       <c r="A159" s="7" t="s">
         <v>185</v>
       </c>
@@ -4469,7 +4479,7 @@
       </c>
       <c r="F159" s="27"/>
     </row>
-    <row r="160" spans="1:6">
+    <row r="160" spans="1:6" hidden="1">
       <c r="A160" s="5" t="s">
         <v>186</v>
       </c>
@@ -4483,7 +4493,7 @@
       <c r="E160" s="26"/>
       <c r="F160" s="27"/>
     </row>
-    <row r="161" spans="1:6">
+    <row r="161" spans="1:6" hidden="1">
       <c r="A161" s="6" t="s">
         <v>187</v>
       </c>
@@ -4519,7 +4529,7 @@
       </c>
       <c r="F162" s="27"/>
     </row>
-    <row r="163" spans="1:6">
+    <row r="163" spans="1:6" hidden="1">
       <c r="A163" s="6" t="s">
         <v>189</v>
       </c>
@@ -4537,7 +4547,7 @@
       </c>
       <c r="F163" s="27"/>
     </row>
-    <row r="164" spans="1:6">
+    <row r="164" spans="1:6" hidden="1">
       <c r="A164" s="4" t="s">
         <v>190</v>
       </c>
@@ -4555,7 +4565,7 @@
       </c>
       <c r="F164" s="27"/>
     </row>
-    <row r="165" spans="1:6">
+    <row r="165" spans="1:6" hidden="1">
       <c r="A165" s="14" t="s">
         <v>191</v>
       </c>
@@ -4573,7 +4583,7 @@
       </c>
       <c r="F165" s="27"/>
     </row>
-    <row r="166" spans="1:6">
+    <row r="166" spans="1:6" hidden="1">
       <c r="A166" s="9" t="s">
         <v>192</v>
       </c>
@@ -4591,7 +4601,7 @@
       </c>
       <c r="F166" s="27"/>
     </row>
-    <row r="167" spans="1:6">
+    <row r="167" spans="1:6" hidden="1">
       <c r="A167" s="15" t="s">
         <v>193</v>
       </c>
@@ -4609,7 +4619,7 @@
       </c>
       <c r="F167" s="27"/>
     </row>
-    <row r="168" spans="1:6">
+    <row r="168" spans="1:6" hidden="1">
       <c r="A168" s="5" t="s">
         <v>194</v>
       </c>
@@ -4623,7 +4633,7 @@
       <c r="E168" s="26"/>
       <c r="F168" s="27"/>
     </row>
-    <row r="169" spans="1:6">
+    <row r="169" spans="1:6" hidden="1">
       <c r="A169" s="5" t="s">
         <v>195</v>
       </c>
@@ -4655,7 +4665,7 @@
       </c>
       <c r="F170" s="27"/>
     </row>
-    <row r="171" spans="1:6">
+    <row r="171" spans="1:6" hidden="1">
       <c r="A171" s="10" t="s">
         <v>197</v>
       </c>
@@ -4673,7 +4683,7 @@
       </c>
       <c r="F171" s="27"/>
     </row>
-    <row r="172" spans="1:6">
+    <row r="172" spans="1:6" hidden="1">
       <c r="A172" s="4" t="s">
         <v>198</v>
       </c>
@@ -4691,7 +4701,7 @@
       </c>
       <c r="F172" s="27"/>
     </row>
-    <row r="173" spans="1:6">
+    <row r="173" spans="1:6" hidden="1">
       <c r="A173" s="5" t="s">
         <v>199</v>
       </c>
@@ -4705,7 +4715,7 @@
       <c r="E173" s="26"/>
       <c r="F173" s="27"/>
     </row>
-    <row r="174" spans="1:6">
+    <row r="174" spans="1:6" hidden="1">
       <c r="A174" s="11" t="s">
         <v>200</v>
       </c>
@@ -4719,7 +4729,7 @@
       <c r="E174" s="26"/>
       <c r="F174" s="27"/>
     </row>
-    <row r="175" spans="1:6">
+    <row r="175" spans="1:6" hidden="1">
       <c r="A175" s="13" t="s">
         <v>201</v>
       </c>
@@ -4737,7 +4747,7 @@
       </c>
       <c r="F175" s="27"/>
     </row>
-    <row r="176" spans="1:6">
+    <row r="176" spans="1:6" hidden="1">
       <c r="A176" s="6" t="s">
         <v>202</v>
       </c>
@@ -4755,7 +4765,7 @@
       </c>
       <c r="F176" s="27"/>
     </row>
-    <row r="177" spans="1:6">
+    <row r="177" spans="1:6" hidden="1">
       <c r="A177" s="11" t="s">
         <v>203</v>
       </c>
@@ -4769,7 +4779,7 @@
       <c r="E177" s="26"/>
       <c r="F177" s="27"/>
     </row>
-    <row r="178" spans="1:6">
+    <row r="178" spans="1:6" hidden="1">
       <c r="A178" s="13" t="s">
         <v>204</v>
       </c>
@@ -4783,7 +4793,7 @@
       <c r="E178" s="26"/>
       <c r="F178" s="27"/>
     </row>
-    <row r="179" spans="1:6">
+    <row r="179" spans="1:6" hidden="1">
       <c r="A179" s="15" t="s">
         <v>205</v>
       </c>
@@ -4819,7 +4829,7 @@
       </c>
       <c r="F180" s="27"/>
     </row>
-    <row r="181" spans="1:6">
+    <row r="181" spans="1:6" hidden="1">
       <c r="A181" s="14" t="s">
         <v>207</v>
       </c>
@@ -6033,11 +6043,11 @@
         <v>10</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>174</v>
+        <v>142</v>
       </c>
       <c r="C15" s="3" t="str">
         <f>IFERROR(VLOOKUP(RR[[#This Row],[Player Name]],Players!A:D,3,0),"")</f>
-        <v>South Africa</v>
+        <v>Pakistan</v>
       </c>
       <c r="D15" s="3"/>
     </row>
@@ -6046,11 +6056,11 @@
         <v>11</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>188</v>
+        <v>174</v>
       </c>
       <c r="C16" s="3" t="str">
         <f>IFERROR(VLOOKUP(RR[[#This Row],[Player Name]],Players!A:D,3,0),"")</f>
-        <v>New Zealand</v>
+        <v>South Africa</v>
       </c>
       <c r="D16" s="3"/>
     </row>
@@ -6059,11 +6069,11 @@
         <v>12</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="C17" s="3" t="str">
         <f>IFERROR(VLOOKUP(RR[[#This Row],[Player Name]],Players!A:D,3,0),"")</f>
-        <v>South Africa</v>
+        <v>New Zealand</v>
       </c>
       <c r="D17" s="3"/>
     </row>
@@ -6072,11 +6082,11 @@
         <v>13</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>206</v>
+        <v>196</v>
       </c>
       <c r="C18" s="3" t="str">
         <f>IFERROR(VLOOKUP(RR[[#This Row],[Player Name]],Players!A:D,3,0),"")</f>
-        <v>India</v>
+        <v>South Africa</v>
       </c>
       <c r="D18" s="3"/>
     </row>
@@ -6084,10 +6094,12 @@
       <c r="A19" s="3">
         <v>14</v>
       </c>
-      <c r="B19" s="3"/>
+      <c r="B19" s="3" t="s">
+        <v>206</v>
+      </c>
       <c r="C19" s="3" t="str">
         <f>IFERROR(VLOOKUP(RR[[#This Row],[Player Name]],Players!A:D,3,0),"")</f>
-        <v/>
+        <v>India</v>
       </c>
       <c r="D19" s="3"/>
     </row>

</xml_diff>

<commit_message>
Update GD injury replacement
</commit_message>
<xml_diff>
--- a/dwl-fantasy-platform/backend/WWC_Config.xlsx
+++ b/dwl-fantasy-platform/backend/WWC_Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kishan/Downloads/Delulu Leagues/DWL Delulu Women's League/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A490ACC9-F00A-4D73-812D-C8B09ED39343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2C3B7CB5-D92A-4357-8B1D-0F879E422BA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" activeTab="4" xr2:uid="{6957E4A2-D1A9-E849-B61B-E8AC1B9AF357}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" activeTab="2" xr2:uid="{6957E4A2-D1A9-E849-B61B-E8AC1B9AF357}"/>
   </bookViews>
   <sheets>
     <sheet name="Players" sheetId="1" r:id="rId1"/>
@@ -1530,7 +1530,7 @@
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{FF49E610-2074-9448-A682-4CF44B25CCCB}" name="GD" displayName="GD" ref="A5:E23" totalsRowShown="0" headerRowDxfId="49" dataDxfId="48" tableBorderDxfId="47">
   <autoFilter ref="A5:E23" xr:uid="{FF49E610-2074-9448-A682-4CF44B25CCCB}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A6:D23">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A6:E23">
     <sortCondition ref="B5:B23"/>
   </sortState>
   <tableColumns count="5">
@@ -5345,16 +5345,16 @@
         <v>12</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="C17" s="3" t="str">
+        <v>73</v>
+      </c>
+      <c r="C17" s="23" t="str">
         <f>IFERROR(VLOOKUP(GD[[#This Row],[Player Name]],Players!A:D,3,0),"")</f>
-        <v>Scotland</v>
+        <v>India</v>
       </c>
       <c r="D17" s="3"/>
-      <c r="E17" s="23">
+      <c r="E17" s="23" t="str">
         <f>IFERROR(VLOOKUP(GD[[#This Row],[Player Name]],Players!A:F,6,FALSE),"")</f>
-        <v>0</v>
+        <v>Replacement</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="15.75">
@@ -5362,11 +5362,11 @@
         <v>13</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>79</v>
+        <v>164</v>
       </c>
       <c r="C18" s="3" t="str">
         <f>IFERROR(VLOOKUP(GD[[#This Row],[Player Name]],Players!A:D,3,0),"")</f>
-        <v>India</v>
+        <v>Scotland</v>
       </c>
       <c r="D18" s="3"/>
       <c r="E18" s="23">
@@ -5379,16 +5379,16 @@
         <v>14</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C19" s="3" t="str">
         <f>IFERROR(VLOOKUP(GD[[#This Row],[Player Name]],Players!A:D,3,0),"")</f>
         <v>India</v>
       </c>
       <c r="D19" s="3"/>
-      <c r="E19" s="23" t="str">
+      <c r="E19" s="23">
         <f>IFERROR(VLOOKUP(GD[[#This Row],[Player Name]],Players!A:F,6,FALSE),"")</f>
-        <v>Injured</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="15.75">
@@ -5396,16 +5396,16 @@
         <v>15</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="C20" s="3" t="str">
         <f>IFERROR(VLOOKUP(GD[[#This Row],[Player Name]],Players!A:D,3,0),"")</f>
-        <v>England</v>
+        <v>India</v>
       </c>
       <c r="D20" s="3"/>
-      <c r="E20" s="23">
+      <c r="E20" s="23" t="str">
         <f>IFERROR(VLOOKUP(GD[[#This Row],[Player Name]],Players!A:F,6,FALSE),"")</f>
-        <v>0</v>
+        <v>Injured</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="15.75">
@@ -5413,11 +5413,11 @@
         <v>16</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>115</v>
+        <v>62</v>
       </c>
       <c r="C21" s="3" t="str">
         <f>IFERROR(VLOOKUP(GD[[#This Row],[Player Name]],Players!A:D,3,0),"")</f>
-        <v>Netherlands</v>
+        <v>England</v>
       </c>
       <c r="D21" s="3"/>
       <c r="E21" s="23">
@@ -5430,11 +5430,11 @@
         <v>17</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>64</v>
+        <v>115</v>
       </c>
       <c r="C22" s="3" t="str">
         <f>IFERROR(VLOOKUP(GD[[#This Row],[Player Name]],Players!A:D,3,0),"")</f>
-        <v>England</v>
+        <v>Netherlands</v>
       </c>
       <c r="D22" s="3"/>
       <c r="E22" s="23">
@@ -5446,15 +5446,17 @@
       <c r="A23" s="3">
         <v>18</v>
       </c>
-      <c r="B23" s="3"/>
-      <c r="C23" s="23" t="str">
+      <c r="B23" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C23" s="3" t="str">
         <f>IFERROR(VLOOKUP(GD[[#This Row],[Player Name]],Players!A:D,3,0),"")</f>
-        <v/>
+        <v>England</v>
       </c>
       <c r="D23" s="3"/>
-      <c r="E23" s="23" t="str">
+      <c r="E23" s="23">
         <f>IFERROR(VLOOKUP(GD[[#This Row],[Player Name]],Players!A:F,6,FALSE),"")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -6086,31 +6088,31 @@
     </row>
     <row r="15" spans="1:5" ht="15.75">
       <c r="A15" s="3">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>73</v>
+        <v>177</v>
       </c>
       <c r="C15" s="3" t="str">
         <f>IFERROR(VLOOKUP(KQ[[#This Row],[Player Name]],Players!A:D,3,0),"")</f>
-        <v>India</v>
+        <v>South Africa</v>
       </c>
       <c r="D15" s="3"/>
-      <c r="E15" s="3" t="str">
+      <c r="E15" s="3">
         <f>IFERROR(VLOOKUP(KQ[[#This Row],[Player Name]],Players!A:F,6,FALSE),"")</f>
-        <v>Replacement</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="15.75">
       <c r="A16" s="3">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>177</v>
+        <v>82</v>
       </c>
       <c r="C16" s="3" t="str">
         <f>IFERROR(VLOOKUP(KQ[[#This Row],[Player Name]],Players!A:D,3,0),"")</f>
-        <v>South Africa</v>
+        <v>India</v>
       </c>
       <c r="D16" s="3"/>
       <c r="E16" s="3">
@@ -6120,16 +6122,18 @@
     </row>
     <row r="17" spans="1:5" ht="15.75">
       <c r="A17" s="3">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="C17" s="3" t="str">
         <f>IFERROR(VLOOKUP(KQ[[#This Row],[Player Name]],Players!A:D,3,0),"")</f>
-        <v>India</v>
-      </c>
-      <c r="D17" s="3"/>
+        <v>England</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>226</v>
+      </c>
       <c r="E17" s="3">
         <f>IFERROR(VLOOKUP(KQ[[#This Row],[Player Name]],Players!A:F,6,FALSE),"")</f>
         <v>0</v>
@@ -6137,18 +6141,16 @@
     </row>
     <row r="18" spans="1:5" ht="15.75">
       <c r="A18" s="3">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C18" s="3" t="str">
+        <v>31</v>
+      </c>
+      <c r="C18" s="23" t="str">
         <f>IFERROR(VLOOKUP(KQ[[#This Row],[Player Name]],Players!A:D,3,0),"")</f>
-        <v>England</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>226</v>
-      </c>
+        <v>Australia</v>
+      </c>
+      <c r="D18" s="3"/>
       <c r="E18" s="3">
         <f>IFERROR(VLOOKUP(KQ[[#This Row],[Player Name]],Players!A:F,6,FALSE),"")</f>
         <v>0</v>
@@ -6156,19 +6158,17 @@
     </row>
     <row r="19" spans="1:5" ht="15.75">
       <c r="A19" s="3">
-        <v>13</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C19" s="23" t="str">
+        <v>14</v>
+      </c>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3" t="str">
         <f>IFERROR(VLOOKUP(KQ[[#This Row],[Player Name]],Players!A:D,3,0),"")</f>
-        <v>Australia</v>
+        <v/>
       </c>
       <c r="D19" s="3"/>
-      <c r="E19" s="3">
+      <c r="E19" s="3" t="str">
         <f>IFERROR(VLOOKUP(KQ[[#This Row],[Player Name]],Players!A:F,6,FALSE),"")</f>
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="20" spans="1:5" ht="15.75">

</xml_diff>